<commit_message>
Add grouped invested capital, company/LP detail pages, import modal
</commit_message>
<xml_diff>
--- a/public/templates/lp_import_template.xlsx
+++ b/public/templates/lp_import_template.xlsx
@@ -42,8 +42,7 @@
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -101,10 +100,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -472,34 +471,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>* = Required field  |  Blue = Required  |  Gray = Optional  |  Do not modify column headers</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
+          <t>* = Required  |  Blue = Required  |  Gray = Optional  |  Called Capital &amp; Distributions: enter existing balances when migrating from another system</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Investor Name*</t>
@@ -522,55 +523,65 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
+          <t>Called Capital</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Distributions</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
           <t>Commitment Date</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Address Line 1</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Address Line 2</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>ZIP Code</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Contact Name</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -595,59 +606,65 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>15/01/2024</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>john@smithfamily.com</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>+1 (415) 555-0100</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>123 Main Street</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Suite 100</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>California</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>94105</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>John Smith</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>Lead investor</t>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>Lead investor — 2 calls made so far</t>
         </is>
       </c>
     </row>
@@ -666,49 +683,120 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>01/03/2024</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>raj@example.com</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>+91 98765 43210</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Plot 12, Koramangala</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Bangalore</t>
         </is>
       </c>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="inlineStr">
         <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
           <t>560034</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>Fully called, partial distribution received</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>New LP - No calls yet</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n">
+        <v>500000</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>newlp@example.com</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>+1 (650) 555-0200</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>78701</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>Committed but no capital called yet</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -720,16 +808,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Field</t>
@@ -742,16 +829,11 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Example</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>Description / Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Investor Name</t>
@@ -767,13 +849,8 @@
           <t>Full legal name of the LP</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Smith Family Office</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Investing As</t>
@@ -786,16 +863,11 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Legal entity name they invest through</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Smith Family Trust</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Legal entity they invest through (trust, LLC, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Commitment Amount</t>
@@ -808,16 +880,11 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Total pledged amount as a number</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>5000000</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Total pledged amount — number only, e.g. 5000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Currency</t>
@@ -830,254 +897,228 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Three-letter currency code</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>USD, EUR, GBP, INR, SGD, AED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
+          <t>Called Capital</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Total already called from this LP. Leave blank for new LPs. Used when migrating existing data — creates an opening balance transaction automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Distributions</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Total already distributed back to this LP. Leave blank if none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
           <t>Commitment Date</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Date of commitment (dd/mm/yyyy)</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>15/01/2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Primary contact email</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>john@smithfamily.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Phone number with country code</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>+1 (415) 555-0100</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Phone with country code, e.g. +1 (415) 555-0100</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Address Line 1</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Street address</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>123 Main Street</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Address Line 2</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Suite, apt, floor etc.</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Suite 100</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Suite, apt, floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>State or province</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>California</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>ZIP Code</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Postal/ZIP code</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>94105</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Postal / ZIP code</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Country name</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Country name, e.g. USA, India</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Contact Name</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Primary contact person name</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>John Smith</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Any additional notes</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Lead investor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixing LP impoet template
</commit_message>
<xml_diff>
--- a/public/templates/lp_import_template.xlsx
+++ b/public/templates/lp_import_template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,25 +27,50 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <i val="1"/>
-      <color rgb="009b9890"/>
+      <color rgb="00666666"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00444444"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00CC0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00666666"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,16 +84,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006b6860"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4F3EF"/>
+        <fgColor rgb="00A0A0A0"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -76,36 +96,27 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,36 +482,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>* = Required  |  Blue = Required  |  Gray = Optional  |  Called Capital &amp; Distributions: enter existing balances when migrating from another system</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Investor Name*</t>
@@ -508,295 +520,291 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Investing As</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+          <t>Investor Type</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Entity Name</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Commitment Amount*</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Currency*</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Called Capital</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Distributions</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Commitment Date</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>GP Contact</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Address Line 1</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Address Line 2</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>ZIP Code</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>Contact Name</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
+    <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Smith Family Office</t>
+          <t>Jack Cheng</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Smith Family Trust</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr"/>
+      <c r="D3" s="4" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n">
-        <v>4000000</v>
-      </c>
       <c r="F3" s="4" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>15/01/2024</t>
-        </is>
-      </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>john@smithfamily.com</t>
+          <t>01/03/2024</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>+1 (415) 555-0100</t>
+          <t>jack@gmail.com</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>123 Main Street</t>
+          <t>408-123-5678</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Suite 100</t>
+          <t>Mohan Verma</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>California</t>
-        </is>
-      </c>
+          <t>46 Adir Way</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr"/>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>94105</t>
+          <t>Hayward</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>94542</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>John Smith</t>
-        </is>
-      </c>
-      <c r="Q3" s="4" t="inlineStr">
-        <is>
-          <t>Lead investor — 2 calls made so far</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
+      <c r="R3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Raj Patel</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
+          <t>David Family Trust</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Institution</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>David Family Trust</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>250000</v>
-      </c>
       <c r="F4" s="4" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>01/03/2024</t>
-        </is>
+        <v>100000</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>raj@example.com</t>
+          <t>15/06/2024</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>+91 98765 43210</t>
+          <t>david@gmail.com</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Plot 12, Koramangala</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="n"/>
+          <t>510-234-4567</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Kishore Mokada</t>
+        </is>
+      </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Bangalore</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="n"/>
+          <t>245 Main St</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>560034</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="n"/>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>95112</t>
+        </is>
+      </c>
       <c r="Q4" s="4" t="inlineStr">
         <is>
-          <t>Fully called, partial distribution received</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>New LP - No calls yet</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n">
+          <t>New LP</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="n">
         <v>500000</v>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>10/05/2026</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>newlp@example.com</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>+1 (650) 555-0200</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="n"/>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>Texas</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>78701</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr"/>
+      <c r="P5" s="4" t="inlineStr"/>
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="4" t="inlineStr">
-        <is>
-          <t>Committed but no capital called yet</t>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>Committed but not yet called</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -808,18 +816,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>Column</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
@@ -833,292 +841,305 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Investor Name</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
+          <t>Investor Name*</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>Full legal name of the LP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Full name of the investor (individual or primary contact for entities).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Investing As</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Legal entity they invest through (trust, LLC, etc.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
+          <t>Investor Type</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>One of: Individual, Institution, Family Office, Corporate. Defaults to Individual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Commitment Amount</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+          <t>Entity Name</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Required if Investor Type is Institution/Family Office/Corporate. Legal entity name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Commitment Amount*</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Total pledged amount — number only, e.g. 5000000</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Total commitment in USD (numbers only, no $ sign). E.g. 100000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Currency*</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>USD, EUR, GBP, INR, SGD, AED</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Use USD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Called Capital</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Total already called from this LP. Leave blank for new LPs. Used when migrating existing data — creates an opening balance transaction automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Amount already called. Leave blank for new LPs with no prior calls. Creates an opening balance transaction when importing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Distributions</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Total already distributed back to this LP. Leave blank if none.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Total distributions received to date. Leave blank if none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Commitment Date</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Date of commitment (dd/mm/yyyy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Format: DD/MM/YYYY or YYYY-MM-DD. E.g. 01/03/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Primary contact email</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Investor email address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Phone with country code, e.g. +1 (415) 555-0100</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Include country code. E.g. +1 (415) 555-0100</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>GP Contact</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Name of the GP who sourced this LP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Address Line 1</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Street address</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Street address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Address Line 2</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Suite, apt, floor</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Suite, apt, floor etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>City</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>State or province</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Full name or abbreviation. E.g. California or CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>ZIP Code</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Postal / ZIP code</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Postal / ZIP code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Country name, e.g. USA, India</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Contact Name</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Primary contact person name</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Defaults to USA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Any additional notes</t>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Any additional notes about this investor.</t>
         </is>
       </c>
     </row>

</xml_diff>